<commit_message>
운동프로그램 갱신 2026-08-01  1:14:33.47
</commit_message>
<xml_diff>
--- a/운동프로그램_재편_v14.xlsx
+++ b/운동프로그램_재편_v14.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_148EEDE9F63BFAE9F2A31C48984BBC82CDA4EADC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C59D599-2997-4763-BA96-A93E7EA38BE7}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_148EEDE9F63BFAE9F2A31C48984BBC82CDA4EADC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{345D1AF2-535D-40C8-A7BD-9BDBDBBA8653}"/>
   <bookViews>
-    <workbookView xWindow="6690" yWindow="1635" windowWidth="29670" windowHeight="18480" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6690" yWindow="1635" windowWidth="29670" windowHeight="18480" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -15930,6 +15930,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -18392,7 +18396,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="276" customHeight="1">
+    <row r="19" spans="1:9" ht="77.25" customHeight="1">
       <c r="A19" s="6" t="s">
         <v>114</v>
       </c>
@@ -18421,7 +18425,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="300" customHeight="1">
+    <row r="20" spans="1:9" ht="48" customHeight="1">
       <c r="A20" s="26">
         <v>1</v>
       </c>
@@ -18451,7 +18455,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="252" customHeight="1">
+    <row r="21" spans="1:9" ht="43.5" customHeight="1">
       <c r="A21" s="7">
         <v>2</v>
       </c>
@@ -18480,7 +18484,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="240" customHeight="1">
+    <row r="22" spans="1:9" ht="48.75" customHeight="1">
       <c r="A22" s="7">
         <v>3</v>
       </c>
@@ -18507,7 +18511,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="212.25" customHeight="1">
+    <row r="23" spans="1:9" ht="33.75" customHeight="1">
       <c r="A23" s="7">
         <v>4</v>
       </c>
@@ -18563,7 +18567,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="105" customHeight="1">
+    <row r="25" spans="1:9" ht="38.25" customHeight="1">
       <c r="D25" s="30" t="s">
         <v>146</v>
       </c>
@@ -20328,7 +20332,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="228" customHeight="1">
+    <row r="19" spans="1:9" ht="49.5" customHeight="1">
       <c r="D19" s="30" t="s">
         <v>146</v>
       </c>

</xml_diff>